<commit_message>
package 18 typos fixed
</commit_message>
<xml_diff>
--- a/curation/draft/cdisc_biomedical_concepts_r18_draft.xlsx
+++ b/curation/draft/cdisc_biomedical_concepts_r18_draft.xlsx
@@ -528,7 +528,7 @@
     <row r="1" ht="57.95" customHeight="1" s="14">
       <c r="A1" s="15" t="inlineStr">
         <is>
-          <t>This spreadsheet contains CDISC Biomedical Concepts loaded from 156 YAML files to be released on 2026-08-25.
+          <t>This spreadsheet contains CDISC Biomedical Concepts loaded from 156 YAML files to be released on 2026-07-14.
 The spreadsheet contains 156 unique CDISC Biomedical Concepts.
 The image on the right shows the relation between Biomedical Concepts and SDTM Dataset Specializations.
 Only a few attributes are shown in the image.</t>
@@ -1425,7 +1425,7 @@
       </c>
       <c r="F9" s="21" t="inlineStr">
         <is>
-          <t>QRS;Clinical or Research Assessment Classification;AJCC Cancer Staging Manual 7th Edition Clincal Classification;AJCC V7;AJCC V7 Clinical Classification Question</t>
+          <t>QRS;Clinical or Research Assessment Classification;AJCC Cancer Staging Manual 7th Edition Clinical Classification;AJCC V7;AJCC V7 Clinical Classification Question</t>
         </is>
       </c>
       <c r="G9" s="20" t="inlineStr">
@@ -1492,7 +1492,7 @@
       </c>
       <c r="F10" s="21" t="inlineStr">
         <is>
-          <t>QRS;Clinical or Research Assessment Classification;AJCC Cancer Staging Manual 7th Edition Clincal Classification;AJCC V7;AJCC V7 Clinical Classification Question</t>
+          <t>QRS;Clinical or Research Assessment Classification;AJCC Cancer Staging Manual 7th Edition Clinical Classification;AJCC V7;AJCC V7 Clinical Classification Question</t>
         </is>
       </c>
       <c r="G10" s="20" t="inlineStr">
@@ -1563,7 +1563,7 @@
       </c>
       <c r="F11" s="21" t="inlineStr">
         <is>
-          <t>QRS;Clinical or Research Assessment Classification;AJCC Cancer Staging Manual 7th Edition Clincal Classification;AJCC V7;AJCC V7 Clinical Classification Question</t>
+          <t>QRS;Clinical or Research Assessment Classification;AJCC Cancer Staging Manual 7th Edition Clinical Classification;AJCC V7;AJCC V7 Clinical Classification Question</t>
         </is>
       </c>
       <c r="G11" s="20" t="inlineStr">
@@ -1630,7 +1630,7 @@
       </c>
       <c r="F12" s="21" t="inlineStr">
         <is>
-          <t>QRS;Clinical or Research Assessment Classification;AJCC Cancer Staging Manual 7th Edition Clincal Classification;AJCC V7;AJCC V7 Clinical Classification Question</t>
+          <t>QRS;Clinical or Research Assessment Classification;AJCC Cancer Staging Manual 7th Edition Clinical Classification;AJCC V7;AJCC V7 Clinical Classification Question</t>
         </is>
       </c>
       <c r="G12" s="20" t="inlineStr">
@@ -1701,7 +1701,7 @@
       </c>
       <c r="F13" s="21" t="inlineStr">
         <is>
-          <t>QRS;Clinical or Research Assessment Classification;AJCC Cancer Staging Manual 7th Edition Clincal Classification;AJCC V7;AJCC V7 Clinical Classification Question</t>
+          <t>QRS;Clinical or Research Assessment Classification;AJCC Cancer Staging Manual 7th Edition Clinical Classification;AJCC V7;AJCC V7 Clinical Classification Question</t>
         </is>
       </c>
       <c r="G13" s="20" t="inlineStr">
@@ -1772,7 +1772,7 @@
       </c>
       <c r="F14" s="21" t="inlineStr">
         <is>
-          <t>QRS;Clinical or Research Assessment Classification;AJCC Cancer Staging Manual 7th Edition Clincal Classification;AJCC V7;AJCC V7 Clinical Classification Question</t>
+          <t>QRS;Clinical or Research Assessment Classification;AJCC Cancer Staging Manual 7th Edition Clinical Classification;AJCC V7;AJCC V7 Clinical Classification Question</t>
         </is>
       </c>
       <c r="G14" s="20" t="inlineStr">
@@ -1839,7 +1839,7 @@
       </c>
       <c r="F15" s="21" t="inlineStr">
         <is>
-          <t>QRS;Clinical or Research Assessment Classification;AJCC Cancer Staging Manual 7th Edition Clincal Classification;AJCC V7;AJCC V7 Clinical Classification Question</t>
+          <t>QRS;Clinical or Research Assessment Classification;AJCC Cancer Staging Manual 7th Edition Clinical Classification;AJCC V7;AJCC V7 Clinical Classification Question</t>
         </is>
       </c>
       <c r="G15" s="20" t="inlineStr">
@@ -1910,7 +1910,7 @@
       </c>
       <c r="F16" s="21" t="inlineStr">
         <is>
-          <t>QRS;Clinical or Research Assessment Classification;AJCC Cancer Staging Manual 7th Edition Clincal Classification;AJCC V7;AJCC V7 Clinical Classification Question</t>
+          <t>QRS;Clinical or Research Assessment Classification;AJCC Cancer Staging Manual 7th Edition Clinical Classification;AJCC V7;AJCC V7 Clinical Classification Question</t>
         </is>
       </c>
       <c r="G16" s="20" t="inlineStr">
@@ -1981,7 +1981,7 @@
       </c>
       <c r="F17" s="21" t="inlineStr">
         <is>
-          <t>QRS;Clinical or Research Assessment Classification;AJCC Cancer Staging Manual 7th Edition Clincal Classification;AJCC V7;AJCC V7 Clinical Classification Question</t>
+          <t>QRS;Clinical or Research Assessment Classification;AJCC Cancer Staging Manual 7th Edition Clinical Classification;AJCC V7;AJCC V7 Clinical Classification Question</t>
         </is>
       </c>
       <c r="G17" s="20" t="inlineStr">
@@ -2048,7 +2048,7 @@
       </c>
       <c r="F18" s="21" t="inlineStr">
         <is>
-          <t>QRS;Clinical or Research Assessment Classification;AJCC Cancer Staging Manual 7th Edition Clincal Classification;AJCC V7;AJCC V7 Clinical Classification Question</t>
+          <t>QRS;Clinical or Research Assessment Classification;AJCC Cancer Staging Manual 7th Edition Clinical Classification;AJCC V7;AJCC V7 Clinical Classification Question</t>
         </is>
       </c>
       <c r="G18" s="20" t="inlineStr">
@@ -2119,7 +2119,7 @@
       </c>
       <c r="F19" s="21" t="inlineStr">
         <is>
-          <t>QRS;Clinical or Research Assessment Classification;AJCC Cancer Staging Manual 7th Edition Clincal Classification;AJCC V7;AJCC V7 Clinical Classification Question</t>
+          <t>QRS;Clinical or Research Assessment Classification;AJCC Cancer Staging Manual 7th Edition Clinical Classification;AJCC V7;AJCC V7 Clinical Classification Question</t>
         </is>
       </c>
       <c r="G19" s="20" t="inlineStr"/>
@@ -2182,7 +2182,7 @@
       </c>
       <c r="F20" s="21" t="inlineStr">
         <is>
-          <t>QRS;Clinical or Research Assessment Classification;AJCC Cancer Staging Manual 7th Edition Clincal Classification;AJCC V7;AJCC V7 Clinical Classification Question</t>
+          <t>QRS;Clinical or Research Assessment Classification;AJCC Cancer Staging Manual 7th Edition Clinical Classification;AJCC V7;AJCC V7 Clinical Classification Question</t>
         </is>
       </c>
       <c r="G20" s="20" t="inlineStr"/>
@@ -2245,7 +2245,7 @@
       </c>
       <c r="F21" s="21" t="inlineStr">
         <is>
-          <t>QRS;Clinical or Research Assessment Classification;AJCC Cancer Staging Manual 7th Edition Clincal Classification;AJCC V7;AJCC V7 Clinical Classification Question</t>
+          <t>QRS;Clinical or Research Assessment Classification;AJCC Cancer Staging Manual 7th Edition Clinical Classification;AJCC V7;AJCC V7 Clinical Classification Question</t>
         </is>
       </c>
       <c r="G21" s="20" t="inlineStr"/>
@@ -2312,7 +2312,7 @@
       </c>
       <c r="F22" s="21" t="inlineStr">
         <is>
-          <t>QRS;Clinical or Research Assessment Classification;AJCC Cancer Staging Manual 7th Edition Clincal Classification;AJCC V7;AJCC V7 Clinical Classification Question</t>
+          <t>QRS;Clinical or Research Assessment Classification;AJCC Cancer Staging Manual 7th Edition Clinical Classification;AJCC V7;AJCC V7 Clinical Classification Question</t>
         </is>
       </c>
       <c r="G22" s="20" t="inlineStr"/>
@@ -2379,7 +2379,7 @@
       </c>
       <c r="F23" s="21" t="inlineStr">
         <is>
-          <t>QRS;Clinical or Research Assessment Classification;AJCC Cancer Staging Manual 7th Edition Clincal Classification;AJCC V7;AJCC V7 Clinical Classification Question</t>
+          <t>QRS;Clinical or Research Assessment Classification;AJCC Cancer Staging Manual 7th Edition Clinical Classification;AJCC V7;AJCC V7 Clinical Classification Question</t>
         </is>
       </c>
       <c r="G23" s="20" t="inlineStr"/>
@@ -2446,7 +2446,7 @@
       </c>
       <c r="F24" s="21" t="inlineStr">
         <is>
-          <t>QRS;Clinical or Research Assessment Classification;AJCC Cancer Staging Manual 7th Edition Clincal Classification;AJCC V7;AJCC V7 Clinical Classification Question</t>
+          <t>QRS;Clinical or Research Assessment Classification;AJCC Cancer Staging Manual 7th Edition Clinical Classification;AJCC V7;AJCC V7 Clinical Classification Question</t>
         </is>
       </c>
       <c r="G24" s="20" t="inlineStr">
@@ -2513,7 +2513,7 @@
       </c>
       <c r="F25" s="21" t="inlineStr">
         <is>
-          <t>QRS;Clinical or Research Assessment Classification;AJCC Cancer Staging Manual 7th Edition Clincal Classification;AJCC V7;AJCC V7 Clinical Classification Question</t>
+          <t>QRS;Clinical or Research Assessment Classification;AJCC Cancer Staging Manual 7th Edition Clinical Classification;AJCC V7;AJCC V7 Clinical Classification Question</t>
         </is>
       </c>
       <c r="G25" s="20" t="inlineStr">
@@ -2584,7 +2584,7 @@
       </c>
       <c r="F26" s="21" t="inlineStr">
         <is>
-          <t>QRS;Clinical or Research Assessment Classification;AJCC Cancer Staging Manual 7th Edition Clincal Classification;AJCC V7;AJCC V7 Clinical Classification Question</t>
+          <t>QRS;Clinical or Research Assessment Classification;AJCC Cancer Staging Manual 7th Edition Clinical Classification;AJCC V7;AJCC V7 Clinical Classification Question</t>
         </is>
       </c>
       <c r="G26" s="20" t="inlineStr">
@@ -2651,7 +2651,7 @@
       </c>
       <c r="F27" s="21" t="inlineStr">
         <is>
-          <t>QRS;Clinical or Research Assessment Classification;AJCC Cancer Staging Manual 7th Edition Clincal Classification;AJCC V7;AJCC V7 Clinical Classification Question</t>
+          <t>QRS;Clinical or Research Assessment Classification;AJCC Cancer Staging Manual 7th Edition Clinical Classification;AJCC V7;AJCC V7 Clinical Classification Question</t>
         </is>
       </c>
       <c r="G27" s="20" t="inlineStr">
@@ -2722,7 +2722,7 @@
       </c>
       <c r="F28" s="21" t="inlineStr">
         <is>
-          <t>QRS;Clinical or Research Assessment Classification;AJCC Cancer Staging Manual 7th Edition Clincal Classification;AJCC V7;AJCC V7 Clinical Classification Question</t>
+          <t>QRS;Clinical or Research Assessment Classification;AJCC Cancer Staging Manual 7th Edition Clinical Classification;AJCC V7;AJCC V7 Clinical Classification Question</t>
         </is>
       </c>
       <c r="G28" s="20" t="inlineStr">
@@ -2793,7 +2793,7 @@
       </c>
       <c r="F29" s="21" t="inlineStr">
         <is>
-          <t>QRS;Clinical or Research Assessment Classification;AJCC Cancer Staging Manual 7th Edition Clincal Classification;AJCC V7;AJCC V7 Clinical Classification Question</t>
+          <t>QRS;Clinical or Research Assessment Classification;AJCC Cancer Staging Manual 7th Edition Clinical Classification;AJCC V7;AJCC V7 Clinical Classification Question</t>
         </is>
       </c>
       <c r="G29" s="20" t="inlineStr">
@@ -2864,7 +2864,7 @@
       </c>
       <c r="F30" s="21" t="inlineStr">
         <is>
-          <t>QRS;Clinical or Research Assessment Classification;AJCC Cancer Staging Manual 7th Edition Clincal Classification;AJCC V7;AJCC V7 Clinical Classification Question</t>
+          <t>QRS;Clinical or Research Assessment Classification;AJCC Cancer Staging Manual 7th Edition Clinical Classification;AJCC V7;AJCC V7 Clinical Classification Question</t>
         </is>
       </c>
       <c r="G30" s="20" t="inlineStr">
@@ -2931,7 +2931,7 @@
       </c>
       <c r="F31" s="21" t="inlineStr">
         <is>
-          <t>QRS;Clinical or Research Assessment Classification;AJCC Cancer Staging Manual 7th Edition Clincal Classification;AJCC V7;AJCC V7 Clinical Classification Question</t>
+          <t>QRS;Clinical or Research Assessment Classification;AJCC Cancer Staging Manual 7th Edition Clinical Classification;AJCC V7;AJCC V7 Clinical Classification Question</t>
         </is>
       </c>
       <c r="G31" s="20" t="inlineStr">
@@ -3002,7 +3002,7 @@
       </c>
       <c r="F32" s="21" t="inlineStr">
         <is>
-          <t>QRS;Clinical or Research Assessment Classification;AJCC Cancer Staging Manual 7th Edition Clincal Classification;AJCC V7;AJCC V7 Clinical Classification Question</t>
+          <t>QRS;Clinical or Research Assessment Classification;AJCC Cancer Staging Manual 7th Edition Clinical Classification;AJCC V7;AJCC V7 Clinical Classification Question</t>
         </is>
       </c>
       <c r="G32" s="20" t="inlineStr">
@@ -3073,7 +3073,7 @@
       </c>
       <c r="F33" s="21" t="inlineStr">
         <is>
-          <t>QRS;Clinical or Research Assessment Classification;AJCC Cancer Staging Manual 7th Edition Clincal Classification;AJCC V7;AJCC V7 Clinical Classification Question</t>
+          <t>QRS;Clinical or Research Assessment Classification;AJCC Cancer Staging Manual 7th Edition Clinical Classification;AJCC V7;AJCC V7 Clinical Classification Question</t>
         </is>
       </c>
       <c r="G33" s="20" t="inlineStr">
@@ -39021,7 +39021,7 @@
       </c>
       <c r="Q548" s="21" t="inlineStr">
         <is>
-          <t>FEMAL;MALE;INTERSEX;NOT REPORTED</t>
+          <t>FEMALE;MALE;INTERSEX;NOT REPORTED</t>
         </is>
       </c>
     </row>
@@ -47434,7 +47434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A128"/>
+  <dimension ref="A1:A127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="12.75"/>
   <cols>
     <col width="82.140625" customWidth="1" style="14" min="1" max="1"/>
@@ -47499,838 +47499,831 @@
     <row r="9">
       <c r="A9" s="21" t="inlineStr">
         <is>
-          <t>AJCC Cancer Staging Manual 7th Edition Clincal Classification</t>
+          <t>AJCC Cancer Staging Manual 7th Edition Clinical Classification</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="21" t="inlineStr">
         <is>
-          <t>AJCC Cancer Staging Manual 7th Edition Clinical Classification</t>
+          <t>AJCC V7</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="21" t="inlineStr">
         <is>
-          <t>AJCC V7</t>
+          <t>AJCC V7 Clinical Classification Question</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="21" t="inlineStr">
         <is>
-          <t>AJCC V7 Clinical Classification Question</t>
+          <t>AJCC1</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="21" t="inlineStr">
         <is>
-          <t>AJCC1</t>
+          <t>AJCC7</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="21" t="inlineStr">
         <is>
-          <t>AJCC7</t>
+          <t>APACHE II</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="21" t="inlineStr">
         <is>
-          <t>APACHE II</t>
+          <t>APCH1</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="21" t="inlineStr">
         <is>
-          <t>APCH1</t>
+          <t>ATLAS</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="21" t="inlineStr">
         <is>
-          <t>ATLAS</t>
+          <t>ATLAS Score Clinical Classification</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="21" t="inlineStr">
         <is>
-          <t>ATLAS Score Clinical Classification</t>
+          <t>ATLAS1</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="21" t="inlineStr">
         <is>
-          <t>ATLAS1</t>
+          <t>Abnormal Involuntary Movement Scale Clinical Classification</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="21" t="inlineStr">
         <is>
-          <t>Abnormal Involuntary Movement Scale Clinical Classification</t>
+          <t>Acute Physiology and Chronic Health Evaluation II Clinical Classification</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="21" t="inlineStr">
         <is>
-          <t>Acute Physiology and Chronic Health Evaluation II Clinical Classification</t>
+          <t>Alzheimer's Disease Assessment Scale-Cognitive CDISC Version Functional Test</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="21" t="inlineStr">
         <is>
-          <t>Alzheimer's Disease Assessment Scale-Cognitive CDISC Version Functional Test</t>
+          <t>BPRS-A</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="21" t="inlineStr">
         <is>
-          <t>BPRS-A</t>
+          <t>BPRSA1</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="21" t="inlineStr">
         <is>
-          <t>BPRSA1</t>
+          <t>Behaviors</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="21" t="inlineStr">
         <is>
-          <t>Behaviors</t>
+          <t>Breast Cancer Procedures</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="21" t="inlineStr">
         <is>
-          <t>Breast Cancer Procedures</t>
+          <t>Brief Psychiatric Rating Scale A Clinical Classification</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="21" t="inlineStr">
         <is>
-          <t>Brief Psychiatric Rating Scale A Clinical Classification</t>
+          <t>CES</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="21" t="inlineStr">
         <is>
-          <t>CES</t>
+          <t>CES01</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="21" t="inlineStr">
         <is>
-          <t>CES01</t>
+          <t>CGI</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="21" t="inlineStr">
         <is>
-          <t>CGI</t>
+          <t>CGI02</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="21" t="inlineStr">
         <is>
-          <t>CGI02</t>
+          <t>CHILD-PUGH CLASSIFICATION</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="21" t="inlineStr">
         <is>
-          <t>CHILD-PUGH CLASSIFICATION</t>
+          <t>CPS01</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="21" t="inlineStr">
         <is>
-          <t>CPS01</t>
+          <t>Chemistry Tests</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="21" t="inlineStr">
         <is>
-          <t>Chemistry Tests</t>
+          <t>Child-Pugh</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="21" t="inlineStr">
         <is>
-          <t>Child-Pugh</t>
+          <t>Child-Pugh Clinical Classification</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="21" t="inlineStr">
         <is>
-          <t>Child-Pugh Clinical Classification</t>
+          <t>Child-Pugh Clinical Classification Question</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="21" t="inlineStr">
         <is>
-          <t>Child-Pugh Clinical Classification Question</t>
+          <t>Clinical Global Impression Generic Modification Version Questionnaire</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="21" t="inlineStr">
         <is>
-          <t>Clinical Global Impression Generic Modification Version Questionnaire</t>
+          <t>Clinical Interventions</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="21" t="inlineStr">
         <is>
-          <t>Clinical Interventions</t>
+          <t>Clinical or Research Assessment Classification</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="21" t="inlineStr">
         <is>
-          <t>Clinical or Research Assessment Classification</t>
+          <t>Clinical or Research Assessment Questionnaire</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="21" t="inlineStr">
         <is>
-          <t>Clinical or Research Assessment Questionnaire</t>
+          <t>Combat Exposure Scale Questionnaire</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="21" t="inlineStr">
         <is>
-          <t>Combat Exposure Scale Questionnaire</t>
+          <t>Contact Information</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="21" t="inlineStr">
         <is>
-          <t>Contact Information</t>
+          <t>Diagnostic Factors</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="21" t="inlineStr">
         <is>
-          <t>Diagnostic Factors</t>
+          <t>Diagnostic Imaging</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="21" t="inlineStr">
         <is>
-          <t>Diagnostic Imaging</t>
+          <t>Diagnostic Procedure</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="21" t="inlineStr">
         <is>
-          <t>Diagnostic Procedure</t>
+          <t>Dietary Mineral Measurements</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="21" t="inlineStr">
         <is>
-          <t>Dietary Mineral Measurements</t>
+          <t>Disease Response</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="21" t="inlineStr">
         <is>
-          <t>Disease Response</t>
+          <t>ECOG</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="21" t="inlineStr">
         <is>
-          <t>ECOG</t>
+          <t>ECOG1</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="21" t="inlineStr">
         <is>
-          <t>ECOG1</t>
+          <t>EQ-5D-5L</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="21" t="inlineStr">
         <is>
-          <t>EQ-5D-5L</t>
+          <t>EQ5D02</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="21" t="inlineStr">
         <is>
-          <t>EQ5D02</t>
+          <t>Eastern Cooperative Oncology Group Performance Status Clinical Classification</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="21" t="inlineStr">
         <is>
-          <t>Eastern Cooperative Oncology Group Performance Status Clinical Classification</t>
+          <t>Electrolyte Measurements</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="21" t="inlineStr">
         <is>
-          <t>Electrolyte Measurements</t>
+          <t>European Quality of Life Five Dimension Five Level Scale Questionnaire</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="21" t="inlineStr">
         <is>
-          <t>European Quality of Life Five Dimension Five Level Scale Questionnaire</t>
+          <t>Functional Assessment</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="21" t="inlineStr">
         <is>
-          <t>Functional Assessment</t>
+          <t>HAM-A</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="21" t="inlineStr">
         <is>
-          <t>HAM-A</t>
+          <t>HAMA</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="21" t="inlineStr">
         <is>
-          <t>HAMA</t>
+          <t>HAMA1</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="21" t="inlineStr">
         <is>
-          <t>HAMA1</t>
+          <t>HBI</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="21" t="inlineStr">
         <is>
-          <t>HBI</t>
+          <t>HBI01</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="21" t="inlineStr">
         <is>
-          <t>HBI01</t>
+          <t>Hamilton Anxiety Rating Scale Clinical Classification</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="21" t="inlineStr">
         <is>
-          <t>Hamilton Anxiety Rating Scale Clinical Classification</t>
+          <t>Harvey-Bradshaw Index Clinical Classification</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="21" t="inlineStr">
         <is>
-          <t>Harvey-Bradshaw Index Clinical Classification</t>
+          <t>Imaging Procedure</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="21" t="inlineStr">
         <is>
-          <t>Imaging Procedure</t>
+          <t>Immunology Tests</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="21" t="inlineStr">
         <is>
-          <t>Immunology Tests</t>
+          <t>Indicators</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="21" t="inlineStr">
         <is>
-          <t>Indicators</t>
+          <t>Integumentary System Findings</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="21" t="inlineStr">
         <is>
-          <t>Integumentary System Findings</t>
+          <t>Interventions</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="21" t="inlineStr">
         <is>
-          <t>Interventions</t>
+          <t>KFSS</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="21" t="inlineStr">
         <is>
-          <t>KFSS</t>
+          <t>KFSS1</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="21" t="inlineStr">
         <is>
-          <t>KFSS1</t>
+          <t>KPS SCALE</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="21" t="inlineStr">
         <is>
-          <t>KPS SCALE</t>
+          <t>KPSS01</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="21" t="inlineStr">
         <is>
-          <t>KPSS01</t>
+          <t>Karnofsky Performance Status Scale Clinical Classification</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="21" t="inlineStr">
         <is>
-          <t>Karnofsky Performance Status Scale Clinical Classification</t>
+          <t>Kurtzke Functional Systems Scores Clinical Classification</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="21" t="inlineStr">
         <is>
-          <t>Kurtzke Functional Systems Scores Clinical Classification</t>
+          <t>Laboratory Tests</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="21" t="inlineStr">
         <is>
-          <t>Laboratory Tests</t>
+          <t>MVAI</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="21" t="inlineStr">
         <is>
-          <t>MVAI</t>
+          <t>MVAI1</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="21" t="inlineStr">
         <is>
-          <t>MVAI1</t>
+          <t>Medical Conditions</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="21" t="inlineStr">
         <is>
-          <t>Medical Conditions</t>
+          <t>Medical History Events</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="21" t="inlineStr">
         <is>
-          <t>Medical History Events</t>
+          <t>Medical Imaging</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="21" t="inlineStr">
         <is>
-          <t>Medical Imaging</t>
+          <t>Microbiology Tests</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="21" t="inlineStr">
         <is>
-          <t>Microbiology Tests</t>
+          <t>Microscopic Findings</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="21" t="inlineStr">
         <is>
-          <t>Microscopic Findings</t>
+          <t>Modified Van Assche Index Clinical Classification</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="21" t="inlineStr">
         <is>
-          <t>Modified Van Assche Index Clinical Classification</t>
+          <t>Modified Van Assche Index Clinical Classification Question</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="21" t="inlineStr">
         <is>
-          <t>Modified Van Assche Index Clinical Classification Question</t>
+          <t>NM</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="21" t="inlineStr">
         <is>
-          <t>NM</t>
+          <t>Nuclear Medicine</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="21" t="inlineStr">
         <is>
-          <t>Nuclear Medicine</t>
+          <t>Oncology Standards</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="21" t="inlineStr">
         <is>
-          <t>Oncology Standards</t>
+          <t>Operations</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="21" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>PASI FREDRIKSSON</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="21" t="inlineStr">
         <is>
-          <t>PASI FREDRIKSSON</t>
+          <t>PASI03</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="21" t="inlineStr">
         <is>
-          <t>PASI03</t>
+          <t>PGI</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="21" t="inlineStr">
         <is>
-          <t>PGI</t>
+          <t>PGI01</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="21" t="inlineStr">
         <is>
-          <t>PGI01</t>
+          <t>Pathology</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="21" t="inlineStr">
         <is>
-          <t>Pathology</t>
+          <t>Patient Global Impression Generic Modification Version Questionnaire</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="21" t="inlineStr">
         <is>
-          <t>Patient Global Impression Generic Modification Version Questionnaire</t>
+          <t>Person Status</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="21" t="inlineStr">
         <is>
-          <t>Person Status</t>
+          <t>Personal Attributes</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="21" t="inlineStr">
         <is>
-          <t>Personal Attributes</t>
+          <t>Presenting Conditions</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="21" t="inlineStr">
         <is>
-          <t>Presenting Conditions</t>
+          <t>Procedures</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="21" t="inlineStr">
         <is>
-          <t>Procedures</t>
+          <t>Psoriasis Area and Severity Index Fredriksson Version Clinical Classification</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="21" t="inlineStr">
         <is>
-          <t>Psoriasis Area and Severity Index Fredriksson Version Clinical Classification</t>
+          <t>Psoriasis Area and Severity Index Fredriksson Version Clinical Classification Question</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="21" t="inlineStr">
         <is>
-          <t>Psoriasis Area and Severity Index Fredriksson Version Clinical Classification Question</t>
+          <t>QRS</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="21" t="inlineStr">
         <is>
-          <t>QRS</t>
+          <t>QRS Instrument Questions</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="21" t="inlineStr">
         <is>
-          <t>QRS Instrument Questions</t>
+          <t>RS</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="21" t="inlineStr">
         <is>
-          <t>RS</t>
+          <t>RUTG01</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="21" t="inlineStr">
         <is>
-          <t>RUTG01</t>
+          <t>RUTGEERTS SCORE</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="21" t="inlineStr">
         <is>
-          <t>RUTGEERTS SCORE</t>
+          <t>Radiation Therapy</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="21" t="inlineStr">
         <is>
-          <t>Radiation Therapy</t>
+          <t>Reported Events</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="21" t="inlineStr">
         <is>
-          <t>Reported Events</t>
+          <t>Rutgeerts Score Clinical Classification</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="21" t="inlineStr">
         <is>
-          <t>Rutgeerts Score Clinical Classification</t>
+          <t>SIX MINUTE WALK</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="21" t="inlineStr">
         <is>
-          <t>SIX MINUTE WALK</t>
+          <t>SIXMW1</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="21" t="inlineStr">
         <is>
-          <t>SIXMW1</t>
+          <t>Social Circumstances</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="21" t="inlineStr">
         <is>
-          <t>Social Circumstances</t>
+          <t>Socioeconomic Factors</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="21" t="inlineStr">
         <is>
-          <t>Socioeconomic Factors</t>
+          <t>Subject Characteristics</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="21" t="inlineStr">
         <is>
-          <t>Subject Characteristics</t>
+          <t>TANN01</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="21" t="inlineStr">
         <is>
-          <t>TANN01</t>
+          <t>TANN02</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="21" t="inlineStr">
         <is>
-          <t>TANN02</t>
+          <t>TANNER SCALE BOY</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="21" t="inlineStr">
         <is>
-          <t>TANNER SCALE BOY</t>
+          <t>TANNER SCALE GIRL</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="21" t="inlineStr">
         <is>
-          <t>TANNER SCALE GIRL</t>
+          <t>TU</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="21" t="inlineStr">
         <is>
-          <t>TU</t>
+          <t>Tanner Scale Boy Version</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="21" t="inlineStr">
         <is>
-          <t>Tanner Scale Boy Version</t>
+          <t>Tanner Scale Girl Version</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="21" t="inlineStr">
         <is>
-          <t>Tanner Scale Girl Version</t>
+          <t>Tanner Scale-Boy</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="21" t="inlineStr">
         <is>
-          <t>Tanner Scale-Boy</t>
+          <t>Tanner Scale-Boy Clinical Classification Question</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="21" t="inlineStr">
         <is>
-          <t>Tanner Scale-Boy Clinical Classification Question</t>
+          <t>Tanner Scale-Girl</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="21" t="inlineStr">
         <is>
-          <t>Tanner Scale-Girl</t>
+          <t>Tanner Scale-Girl Clinical Classification Question</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="21" t="inlineStr">
         <is>
-          <t>Tanner Scale-Girl Clinical Classification Question</t>
+          <t>Therapeutic Procedure</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="21" t="inlineStr">
         <is>
-          <t>Therapeutic Procedure</t>
+          <t>Tomagraphy</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="21" t="inlineStr">
         <is>
-          <t>Tomagraphy</t>
+          <t>Tumor/Lesion Identification</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="21" t="inlineStr">
-        <is>
-          <t>Tumor/Lesion Identification</t>
-        </is>
-      </c>
-    </row>
-    <row r="128">
-      <c r="A128" s="21" t="inlineStr">
         <is>
           <t>Virology Tests</t>
         </is>
@@ -48591,7 +48584,7 @@
       </c>
       <c r="E5" s="21" t="inlineStr">
         <is>
-          <t>QRS;Clinical or Research Assessment Classification;AJCC Cancer Staging Manual 7th Edition Clincal Classification;AJCC V7;AJCC V7 Clinical Classification Question</t>
+          <t>QRS;Clinical or Research Assessment Classification;AJCC Cancer Staging Manual 7th Edition Clinical Classification;AJCC V7;AJCC V7 Clinical Classification Question</t>
         </is>
       </c>
       <c r="F5" s="20" t="inlineStr">
@@ -48640,7 +48633,7 @@
       </c>
       <c r="E6" s="21" t="inlineStr">
         <is>
-          <t>QRS;Clinical or Research Assessment Classification;AJCC Cancer Staging Manual 7th Edition Clincal Classification;AJCC V7;AJCC V7 Clinical Classification Question</t>
+          <t>QRS;Clinical or Research Assessment Classification;AJCC Cancer Staging Manual 7th Edition Clinical Classification;AJCC V7;AJCC V7 Clinical Classification Question</t>
         </is>
       </c>
       <c r="F6" s="20" t="inlineStr">
@@ -48689,7 +48682,7 @@
       </c>
       <c r="E7" s="21" t="inlineStr">
         <is>
-          <t>QRS;Clinical or Research Assessment Classification;AJCC Cancer Staging Manual 7th Edition Clincal Classification;AJCC V7;AJCC V7 Clinical Classification Question</t>
+          <t>QRS;Clinical or Research Assessment Classification;AJCC Cancer Staging Manual 7th Edition Clinical Classification;AJCC V7;AJCC V7 Clinical Classification Question</t>
         </is>
       </c>
       <c r="F7" s="20" t="inlineStr"/>
@@ -48734,7 +48727,7 @@
       </c>
       <c r="E8" s="21" t="inlineStr">
         <is>
-          <t>QRS;Clinical or Research Assessment Classification;AJCC Cancer Staging Manual 7th Edition Clincal Classification;AJCC V7;AJCC V7 Clinical Classification Question</t>
+          <t>QRS;Clinical or Research Assessment Classification;AJCC Cancer Staging Manual 7th Edition Clinical Classification;AJCC V7;AJCC V7 Clinical Classification Question</t>
         </is>
       </c>
       <c r="F8" s="20" t="inlineStr">
@@ -48783,7 +48776,7 @@
       </c>
       <c r="E9" s="21" t="inlineStr">
         <is>
-          <t>QRS;Clinical or Research Assessment Classification;AJCC Cancer Staging Manual 7th Edition Clincal Classification;AJCC V7;AJCC V7 Clinical Classification Question</t>
+          <t>QRS;Clinical or Research Assessment Classification;AJCC Cancer Staging Manual 7th Edition Clinical Classification;AJCC V7;AJCC V7 Clinical Classification Question</t>
         </is>
       </c>
       <c r="F9" s="20" t="inlineStr">

</xml_diff>